<commit_message>
halo article and points
</commit_message>
<xml_diff>
--- a/Brentuar PK Invitational Season 1.xlsx
+++ b/Brentuar PK Invitational Season 1.xlsx
@@ -9,8 +9,8 @@
     <sheet state="visible" name="Individual Results" sheetId="4" r:id="rId8"/>
     <sheet state="visible" name="Fall Guys Results" sheetId="5" r:id="rId9"/>
     <sheet state="visible" name="Halo Results AOB" sheetId="6" r:id="rId10"/>
-    <sheet state="visible" name="Halo Results LG" sheetId="7" r:id="rId11"/>
-    <sheet state="visible" name="Halo Results OB" sheetId="8" r:id="rId12"/>
+    <sheet state="visible" name="Halo Results OB" sheetId="7" r:id="rId11"/>
+    <sheet state="visible" name="Halo Results TS" sheetId="8" r:id="rId12"/>
     <sheet state="visible" name="Halo Results CTF" sheetId="9" r:id="rId13"/>
     <sheet state="visible" name="Halo Results" sheetId="10" r:id="rId14"/>
     <sheet state="visible" name="Formula 1 Results" sheetId="11" r:id="rId15"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="76">
   <si>
     <t>Team Brentuar</t>
   </si>
@@ -231,6 +231,9 @@
   </si>
   <si>
     <t>Assists</t>
+  </si>
+  <si>
+    <t>Team Total</t>
   </si>
   <si>
     <t>Driver</t>
@@ -979,6 +982,9 @@
       <c r="E1" s="22" t="s">
         <v>56</v>
       </c>
+      <c r="F1" s="22" t="s">
+        <v>68</v>
+      </c>
       <c r="G1" s="22" t="s">
         <v>21</v>
       </c>
@@ -988,23 +994,27 @@
     </row>
     <row r="2">
       <c r="A2" s="22" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="B2" s="23">
-        <f>'Halo Results OB'!B2 + 'Halo Results LG'!B2 + 'Halo Results AOB'!B2 + 'Halo Results CTF'!B2</f>
-        <v>0</v>
+        <f>'Halo Results TS'!B2 + 'Halo Results OB'!B2 + 'Halo Results AOB'!B2 + 'Halo Results CTF'!B2</f>
+        <v>87</v>
       </c>
       <c r="C2" s="23">
-        <f>'Halo Results OB'!C2 + 'Halo Results LG'!C2 + 'Halo Results AOB'!C2 + 'Halo Results CTF'!C2</f>
-        <v>0</v>
+        <f>'Halo Results TS'!C2 + 'Halo Results OB'!C2 + 'Halo Results AOB'!C2 + 'Halo Results CTF'!C2</f>
+        <v>28</v>
       </c>
       <c r="D2" s="23">
-        <f>'Halo Results OB'!D2 + 'Halo Results LG'!D2 + 'Halo Results AOB'!D2 + 'Halo Results CTF'!D2</f>
+        <f>'Halo Results TS'!D2 + 'Halo Results OB'!D2 + 'Halo Results AOB'!D2 + 'Halo Results CTF'!D2</f>
         <v>0</v>
       </c>
       <c r="E2" s="23">
-        <f t="shared" ref="E2:E9" si="1">B2*$H$1 + C2*$H$2 + D2*$H$3</f>
-        <v>0</v>
+        <f>SUM('Halo Results CTF'!E2+'Halo Results TS'!E2+'Halo Results OB'!E2+'Halo Results AOB'!E2)</f>
+        <v>8</v>
+      </c>
+      <c r="F2" s="23">
+        <f>ROUND(SUM(E2:E5),0)</f>
+        <v>23</v>
       </c>
       <c r="G2" s="22" t="s">
         <v>22</v>
@@ -1015,28 +1025,28 @@
     </row>
     <row r="3">
       <c r="A3" s="22" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="B3" s="23">
-        <f>'Halo Results OB'!B3 + 'Halo Results LG'!B3 + 'Halo Results AOB'!B3 + 'Halo Results CTF'!B3</f>
-        <v>0</v>
+        <f>'Halo Results TS'!B3 + 'Halo Results OB'!B3 + 'Halo Results AOB'!B3 + 'Halo Results CTF'!B3</f>
+        <v>35</v>
       </c>
       <c r="C3" s="23">
-        <f>'Halo Results OB'!C3 + 'Halo Results LG'!C3 + 'Halo Results AOB'!C3 + 'Halo Results CTF'!C3</f>
-        <v>0</v>
+        <f>'Halo Results TS'!C3 + 'Halo Results OB'!C3 + 'Halo Results AOB'!C3 + 'Halo Results CTF'!C3</f>
+        <v>27</v>
       </c>
       <c r="D3" s="22">
         <v>0.0</v>
       </c>
       <c r="E3" s="23">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>SUM('Halo Results CTF'!E3+'Halo Results TS'!E3+'Halo Results OB'!E3+'Halo Results AOB'!E3)</f>
+        <v>4</v>
       </c>
       <c r="G3" s="22" t="s">
         <v>20</v>
       </c>
       <c r="H3" s="22">
-        <v>10.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="4">
@@ -1044,19 +1054,19 @@
         <v>16</v>
       </c>
       <c r="B4" s="23">
-        <f>'Halo Results OB'!B4 + 'Halo Results LG'!B4 + 'Halo Results AOB'!B4 + 'Halo Results CTF'!B4</f>
-        <v>0</v>
+        <f>'Halo Results TS'!B4 + 'Halo Results OB'!B4 + 'Halo Results AOB'!B4 + 'Halo Results CTF'!B4</f>
+        <v>39</v>
       </c>
       <c r="C4" s="23">
-        <f>'Halo Results OB'!C4 + 'Halo Results LG'!C4 + 'Halo Results AOB'!C4 + 'Halo Results CTF'!C4</f>
-        <v>0</v>
+        <f>'Halo Results TS'!C4 + 'Halo Results OB'!C4 + 'Halo Results AOB'!C4 + 'Halo Results CTF'!C4</f>
+        <v>20</v>
       </c>
       <c r="D4" s="22">
         <v>0.0</v>
       </c>
       <c r="E4" s="23">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>SUM('Halo Results CTF'!E4+'Halo Results TS'!E4+'Halo Results OB'!E4+'Halo Results AOB'!E4)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -1064,19 +1074,19 @@
         <v>14</v>
       </c>
       <c r="B5" s="25">
-        <f>'Halo Results OB'!B5 + 'Halo Results LG'!B5 + 'Halo Results AOB'!B5 + 'Halo Results CTF'!B5</f>
-        <v>0</v>
+        <f>'Halo Results TS'!B5 + 'Halo Results OB'!B5 + 'Halo Results AOB'!B5 + 'Halo Results CTF'!B5</f>
+        <v>52</v>
       </c>
       <c r="C5" s="25">
-        <f>'Halo Results OB'!C5 + 'Halo Results LG'!C5 + 'Halo Results AOB'!C5 + 'Halo Results CTF'!C5</f>
-        <v>0</v>
+        <f>'Halo Results TS'!C5 + 'Halo Results OB'!C5 + 'Halo Results AOB'!C5 + 'Halo Results CTF'!C5</f>
+        <v>35</v>
       </c>
       <c r="D5" s="24">
         <v>0.0</v>
       </c>
       <c r="E5" s="25">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>SUM('Halo Results CTF'!E5+'Halo Results TS'!E5+'Halo Results OB'!E5+'Halo Results AOB'!E5)</f>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -1084,20 +1094,24 @@
         <v>11</v>
       </c>
       <c r="B6" s="23">
-        <f>'Halo Results OB'!B6 + 'Halo Results LG'!B6 + 'Halo Results AOB'!B6 + 'Halo Results CTF'!B6</f>
-        <v>0</v>
+        <f>'Halo Results TS'!B6 + 'Halo Results OB'!B6 + 'Halo Results AOB'!B6 + 'Halo Results CTF'!B6</f>
+        <v>105</v>
       </c>
       <c r="C6" s="23">
-        <f>'Halo Results OB'!C6 + 'Halo Results LG'!C6 + 'Halo Results AOB'!C6 + 'Halo Results CTF'!C6</f>
-        <v>0</v>
+        <f>'Halo Results TS'!C6 + 'Halo Results OB'!C6 + 'Halo Results AOB'!C6 + 'Halo Results CTF'!C6</f>
+        <v>33</v>
       </c>
       <c r="D6" s="23">
-        <f>'Halo Results OB'!D6 + 'Halo Results LG'!D6 + 'Halo Results AOB'!D6 + 'Halo Results CTF'!D6</f>
-        <v>0</v>
+        <f>'Halo Results TS'!D6 + 'Halo Results OB'!D6 + 'Halo Results AOB'!D6 + 'Halo Results CTF'!D6</f>
+        <v>3</v>
       </c>
       <c r="E6" s="23">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>SUM('Halo Results CTF'!E6+'Halo Results TS'!E6+'Halo Results OB'!E6+'Halo Results AOB'!E6)</f>
+        <v>14</v>
+      </c>
+      <c r="F6" s="23">
+        <f>ROUND(SUM(E6:E9),0)</f>
+        <v>33</v>
       </c>
     </row>
     <row r="7">
@@ -1105,19 +1119,19 @@
         <v>7</v>
       </c>
       <c r="B7" s="23">
-        <f>'Halo Results OB'!B7 + 'Halo Results LG'!B7 + 'Halo Results AOB'!B7 + 'Halo Results CTF'!B7</f>
-        <v>0</v>
+        <f>'Halo Results TS'!B7 + 'Halo Results OB'!B7 + 'Halo Results AOB'!B7 + 'Halo Results CTF'!B7</f>
+        <v>36</v>
       </c>
       <c r="C7" s="23">
-        <f>'Halo Results OB'!C7 + 'Halo Results LG'!C7 + 'Halo Results AOB'!C7 + 'Halo Results CTF'!C7</f>
-        <v>0</v>
+        <f>'Halo Results TS'!C7 + 'Halo Results OB'!C7 + 'Halo Results AOB'!C7 + 'Halo Results CTF'!C7</f>
+        <v>32</v>
       </c>
       <c r="D7" s="22">
         <v>0.0</v>
       </c>
       <c r="E7" s="23">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>SUM('Halo Results CTF'!E7+'Halo Results TS'!E7+'Halo Results OB'!E7+'Halo Results AOB'!E7)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -1125,19 +1139,19 @@
         <v>13</v>
       </c>
       <c r="B8" s="23">
-        <f>'Halo Results OB'!B8 + 'Halo Results LG'!B8 + 'Halo Results AOB'!B8 + 'Halo Results CTF'!B8</f>
-        <v>0</v>
+        <f>'Halo Results TS'!B8 + 'Halo Results OB'!B8 + 'Halo Results AOB'!B8 + 'Halo Results CTF'!B8</f>
+        <v>82</v>
       </c>
       <c r="C8" s="23">
-        <f>'Halo Results OB'!C8 + 'Halo Results LG'!C8 + 'Halo Results AOB'!C8 + 'Halo Results CTF'!C8</f>
-        <v>0</v>
+        <f>'Halo Results TS'!C8 + 'Halo Results OB'!C8 + 'Halo Results AOB'!C8 + 'Halo Results CTF'!C8</f>
+        <v>29</v>
       </c>
       <c r="D8" s="22">
         <v>0.0</v>
       </c>
       <c r="E8" s="23">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>SUM('Halo Results CTF'!E8+'Halo Results TS'!E8+'Halo Results OB'!E8+'Halo Results AOB'!E8)</f>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -1145,19 +1159,19 @@
         <v>17</v>
       </c>
       <c r="B9" s="23">
-        <f>'Halo Results OB'!B9 + 'Halo Results LG'!B9 + 'Halo Results AOB'!B9 + 'Halo Results CTF'!B9</f>
-        <v>0</v>
+        <f>'Halo Results TS'!B9 + 'Halo Results OB'!B9 + 'Halo Results AOB'!B9 + 'Halo Results CTF'!B9</f>
+        <v>49</v>
       </c>
       <c r="C9" s="23">
-        <f>'Halo Results OB'!C9 + 'Halo Results LG'!C9 + 'Halo Results AOB'!C9 + 'Halo Results CTF'!C9</f>
-        <v>0</v>
+        <f>'Halo Results TS'!C9 + 'Halo Results OB'!C9 + 'Halo Results AOB'!C9 + 'Halo Results CTF'!C9</f>
+        <v>16</v>
       </c>
       <c r="D9" s="22">
         <v>0.0</v>
       </c>
       <c r="E9" s="23">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>SUM('Halo Results CTF'!E9+'Halo Results TS'!E9+'Halo Results OB'!E9+'Halo Results AOB'!E9)</f>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1174,7 +1188,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="22" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B1" s="22" t="s">
         <v>38</v>
@@ -1183,13 +1197,13 @@
         <v>39</v>
       </c>
       <c r="D1" s="22" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E1" s="22" t="s">
         <v>40</v>
       </c>
       <c r="F1" s="22" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G1" s="22" t="s">
         <v>47</v>
@@ -1204,16 +1218,16 @@
         <v>56</v>
       </c>
       <c r="L1" s="22" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="M1" s="22" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O1" s="22" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="P1" s="22" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2">
@@ -1745,7 +1759,7 @@
       </c>
       <c r="C2" s="23">
         <f>IF(SUM('Individual Results'!C2:C8)&lt;80,SUM('Individual Results'!C2:C8),80)</f>
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="D2" s="23">
         <f>IF(SUM('Individual Results'!D2:D8)&lt;80,SUM('Individual Results'!D2:D8),80)</f>
@@ -1753,7 +1767,7 @@
       </c>
       <c r="E2" s="23">
         <f t="shared" ref="E2:E3" si="1">SUM(B2:D2)</f>
-        <v>20</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3">
@@ -1766,7 +1780,7 @@
       </c>
       <c r="C3" s="23">
         <f>IF(SUM('Individual Results'!C9:C14)&lt;80,SUM('Individual Results'!C9:C14),80)</f>
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="D3" s="23">
         <f>IF(SUM('Individual Results'!D9:D14)&lt;80,SUM('Individual Results'!D9:D14),80)</f>
@@ -1774,7 +1788,7 @@
       </c>
       <c r="E3" s="23">
         <f t="shared" si="1"/>
-        <v>80</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -1815,8 +1829,8 @@
         <v>0</v>
       </c>
       <c r="C2" s="23">
-        <f t="array" ref="C2">XLOOKUP(A2,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A2,'Halo Results LG'!$A$2:$A$9,'Halo Results LG'!$E$2:$E$9,0) + XLOOKUP(A2,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A2,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
-        <v>0</v>
+        <f t="array" ref="C2">XLOOKUP(A2,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A2,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A2,'Halo Results TS'!$A$2:$A$9,'Halo Results TS'!$E$2:$E$9,0) + XLOOKUP(A2,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
+        <v>4</v>
       </c>
       <c r="D2" s="23">
         <f t="array" ref="D2">XLOOKUP(A2,'Formula 1 Results'!$A$2:$A$9,'Formula 1 Results'!$J$2:$J$9,0)</f>
@@ -1824,7 +1838,7 @@
       </c>
       <c r="E2" s="23">
         <f t="shared" ref="E2:E14" si="1">SUM(B2:D2)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -1836,7 +1850,7 @@
         <v>10</v>
       </c>
       <c r="C3" s="23">
-        <f t="array" ref="C3">XLOOKUP(A3,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A3,'Halo Results LG'!$A$2:$A$9,'Halo Results LG'!$E$2:$E$9,0) + XLOOKUP(A3,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A3,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
+        <f t="array" ref="C3">XLOOKUP(A3,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A3,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A3,'Halo Results TS'!$A$2:$A$9,'Halo Results TS'!$E$2:$E$9,0) + XLOOKUP(A3,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
         <v>0</v>
       </c>
       <c r="D3" s="23">
@@ -1857,7 +1871,7 @@
         <v>10</v>
       </c>
       <c r="C4" s="23">
-        <f t="array" ref="C4">XLOOKUP(A4,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A4,'Halo Results LG'!$A$2:$A$9,'Halo Results LG'!$E$2:$E$9,0) + XLOOKUP(A4,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A4,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
+        <f t="array" ref="C4">XLOOKUP(A4,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A4,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A4,'Halo Results TS'!$A$2:$A$9,'Halo Results TS'!$E$2:$E$9,0) + XLOOKUP(A4,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
         <v>0</v>
       </c>
       <c r="D4" s="23">
@@ -1878,7 +1892,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="23">
-        <f t="array" ref="C5">XLOOKUP(A5,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A5,'Halo Results LG'!$A$2:$A$9,'Halo Results LG'!$E$2:$E$9,0) + XLOOKUP(A5,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A5,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
+        <f t="array" ref="C5">XLOOKUP(A5,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A5,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A5,'Halo Results TS'!$A$2:$A$9,'Halo Results TS'!$E$2:$E$9,0) + XLOOKUP(A5,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
         <v>0</v>
       </c>
       <c r="D5" s="23">
@@ -1899,8 +1913,8 @@
         <v>0</v>
       </c>
       <c r="C6" s="23">
-        <f t="array" ref="C6">XLOOKUP(A6,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A6,'Halo Results LG'!$A$2:$A$9,'Halo Results LG'!$E$2:$E$9,0) + XLOOKUP(A6,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A6,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
-        <v>0</v>
+        <f t="array" ref="C6">XLOOKUP(A6,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A6,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A6,'Halo Results TS'!$A$2:$A$9,'Halo Results TS'!$E$2:$E$9,0) + XLOOKUP(A6,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
+        <v>6</v>
       </c>
       <c r="D6" s="23">
         <f t="array" ref="D6">XLOOKUP(A6,'Formula 1 Results'!$A$2:$A$9,'Formula 1 Results'!$J$2:$J$9,0)</f>
@@ -1908,7 +1922,7 @@
       </c>
       <c r="E6" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -1920,8 +1934,8 @@
         <v>0</v>
       </c>
       <c r="C7" s="23">
-        <f t="array" ref="C7">XLOOKUP(A7,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A7,'Halo Results LG'!$A$2:$A$9,'Halo Results LG'!$E$2:$E$9,0) + XLOOKUP(A7,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A7,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
-        <v>0</v>
+        <f t="array" ref="C7">XLOOKUP(A7,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A7,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A7,'Halo Results TS'!$A$2:$A$9,'Halo Results TS'!$E$2:$E$9,0) + XLOOKUP(A7,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
+        <v>5</v>
       </c>
       <c r="D7" s="23">
         <f t="array" ref="D7">XLOOKUP(A7,'Formula 1 Results'!$A$2:$A$9,'Formula 1 Results'!$J$2:$J$9,0)</f>
@@ -1929,7 +1943,7 @@
       </c>
       <c r="E7" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -1941,8 +1955,8 @@
         <v>0</v>
       </c>
       <c r="C8" s="25">
-        <f t="array" ref="C8">XLOOKUP(A8,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A8,'Halo Results LG'!$A$2:$A$9,'Halo Results LG'!$E$2:$E$9,0) + XLOOKUP(A8,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A8,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
-        <v>0</v>
+        <f t="array" ref="C8">XLOOKUP(A8,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A8,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A8,'Halo Results TS'!$A$2:$A$9,'Halo Results TS'!$E$2:$E$9,0) + XLOOKUP(A8,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
+        <v>8</v>
       </c>
       <c r="D8" s="25">
         <f t="array" ref="D8">XLOOKUP(A8,'Formula 1 Results'!$A$2:$A$9,'Formula 1 Results'!$J$2:$J$9,0)</f>
@@ -1950,7 +1964,7 @@
       </c>
       <c r="E8" s="25">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -1962,8 +1976,8 @@
         <v>0</v>
       </c>
       <c r="C9" s="23">
-        <f t="array" ref="C9">XLOOKUP(A9,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A9,'Halo Results LG'!$A$2:$A$9,'Halo Results LG'!$E$2:$E$9,0) + XLOOKUP(A9,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A9,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
-        <v>0</v>
+        <f t="array" ref="C9">XLOOKUP(A9,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A9,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A9,'Halo Results TS'!$A$2:$A$9,'Halo Results TS'!$E$2:$E$9,0) + XLOOKUP(A9,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
+        <v>5</v>
       </c>
       <c r="D9" s="23">
         <f t="array" ref="D9">XLOOKUP(A9,'Formula 1 Results'!$A$2:$A$9,'Formula 1 Results'!$J$2:$J$9,0)</f>
@@ -1971,7 +1985,7 @@
       </c>
       <c r="E9" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -1983,7 +1997,7 @@
         <v>45</v>
       </c>
       <c r="C10" s="23">
-        <f t="array" ref="C10">XLOOKUP(A10,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A10,'Halo Results LG'!$A$2:$A$9,'Halo Results LG'!$E$2:$E$9,0) + XLOOKUP(A10,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A10,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
+        <f t="array" ref="C10">XLOOKUP(A10,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A10,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A10,'Halo Results TS'!$A$2:$A$9,'Halo Results TS'!$E$2:$E$9,0) + XLOOKUP(A10,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
         <v>0</v>
       </c>
       <c r="D10" s="23">
@@ -2004,8 +2018,8 @@
         <v>10</v>
       </c>
       <c r="C11" s="23">
-        <f t="array" ref="C11">XLOOKUP(A11,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A11,'Halo Results LG'!$A$2:$A$9,'Halo Results LG'!$E$2:$E$9,0) + XLOOKUP(A11,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A11,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
-        <v>0</v>
+        <f t="array" ref="C11">XLOOKUP(A11,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A11,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A11,'Halo Results TS'!$A$2:$A$9,'Halo Results TS'!$E$2:$E$9,0) + XLOOKUP(A11,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
+        <v>14</v>
       </c>
       <c r="D11" s="23">
         <f t="array" ref="D11">XLOOKUP(A11,'Formula 1 Results'!$A$2:$A$9,'Formula 1 Results'!$J$2:$J$9,0)</f>
@@ -2013,7 +2027,7 @@
       </c>
       <c r="E11" s="23">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12">
@@ -2025,8 +2039,8 @@
         <v>85</v>
       </c>
       <c r="C12" s="23">
-        <f t="array" ref="C12">XLOOKUP(A12,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A12,'Halo Results LG'!$A$2:$A$9,'Halo Results LG'!$E$2:$E$9,0) + XLOOKUP(A12,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A12,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
-        <v>0</v>
+        <f t="array" ref="C12">XLOOKUP(A12,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A12,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A12,'Halo Results TS'!$A$2:$A$9,'Halo Results TS'!$E$2:$E$9,0) + XLOOKUP(A12,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
+        <v>9</v>
       </c>
       <c r="D12" s="23">
         <f t="array" ref="D12">XLOOKUP(A12,'Formula 1 Results'!$A$2:$A$9,'Formula 1 Results'!$J$2:$J$9,0)</f>
@@ -2034,7 +2048,7 @@
       </c>
       <c r="E12" s="23">
         <f t="shared" si="1"/>
-        <v>85</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13">
@@ -2046,7 +2060,7 @@
         <v>0</v>
       </c>
       <c r="C13" s="23">
-        <f t="array" ref="C13">XLOOKUP(A13,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A13,'Halo Results LG'!$A$2:$A$9,'Halo Results LG'!$E$2:$E$9,0) + XLOOKUP(A13,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A13,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
+        <f t="array" ref="C13">XLOOKUP(A13,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A13,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A13,'Halo Results TS'!$A$2:$A$9,'Halo Results TS'!$E$2:$E$9,0) + XLOOKUP(A13,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
         <v>0</v>
       </c>
       <c r="D13" s="23">
@@ -2067,8 +2081,8 @@
         <v>0</v>
       </c>
       <c r="C14" s="23">
-        <f t="array" ref="C14">XLOOKUP(A14,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A14,'Halo Results LG'!$A$2:$A$9,'Halo Results LG'!$E$2:$E$9,0) + XLOOKUP(A14,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A14,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
-        <v>0</v>
+        <f t="array" ref="C14">XLOOKUP(A14,'Halo Results AOB'!$A$2:$A$9,'Halo Results AOB'!$E$2:$E$9,0) + XLOOKUP(A14,'Halo Results OB'!$A$2:$A$9,'Halo Results OB'!$E$2:$E$9,0) + XLOOKUP(A14,'Halo Results TS'!$A$2:$A$9,'Halo Results TS'!$E$2:$E$9,0) + XLOOKUP(A14,'Halo Results CTF'!$A$2:$A$9,'Halo Results CTF'!$E$2:$E$9,0)</f>
+        <v>5</v>
       </c>
       <c r="D14" s="23">
         <f t="array" ref="D14">XLOOKUP(A14,'Formula 1 Results'!$A$2:$A$9,'Formula 1 Results'!$J$2:$J$9,0)</f>
@@ -2076,7 +2090,7 @@
       </c>
       <c r="E14" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -2279,6 +2293,9 @@
       <c r="E1" s="22" t="s">
         <v>56</v>
       </c>
+      <c r="F1" s="22" t="s">
+        <v>68</v>
+      </c>
       <c r="G1" s="22" t="s">
         <v>21</v>
       </c>
@@ -2288,11 +2305,24 @@
     </row>
     <row r="2">
       <c r="A2" s="22" t="s">
-        <v>5</v>
+        <v>18</v>
+      </c>
+      <c r="B2" s="22">
+        <v>21.0</v>
+      </c>
+      <c r="C2" s="22">
+        <v>10.0</v>
+      </c>
+      <c r="D2" s="22">
+        <v>0.0</v>
       </c>
       <c r="E2" s="23">
-        <f t="shared" ref="E2:E9" si="1">B2*$H$1 + C2*$H$2 + D2*$H$3</f>
-        <v>0</v>
+        <f t="shared" ref="E2:E9" si="1">ROUND(B2*$H$1 + C2*$H$2 + D2*$H$3,0)</f>
+        <v>2</v>
+      </c>
+      <c r="F2" s="23">
+        <f>SUM(E2:E5)</f>
+        <v>6</v>
       </c>
       <c r="G2" s="22" t="s">
         <v>22</v>
@@ -2303,91 +2333,138 @@
     </row>
     <row r="3">
       <c r="A3" s="22" t="s">
-        <v>18</v>
+        <v>5</v>
+      </c>
+      <c r="B3" s="22">
+        <v>19.0</v>
+      </c>
+      <c r="C3" s="22">
+        <v>10.0</v>
       </c>
       <c r="D3" s="22">
         <v>0.0</v>
       </c>
       <c r="E3" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G3" s="22" t="s">
         <v>20</v>
       </c>
       <c r="H3" s="22">
-        <v>10.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="22" t="s">
         <v>16</v>
       </c>
+      <c r="B4" s="22">
+        <v>9.0</v>
+      </c>
+      <c r="C4" s="22">
+        <v>5.0</v>
+      </c>
       <c r="D4" s="22">
         <v>0.0</v>
       </c>
       <c r="E4" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
+      <c r="B5" s="24">
+        <v>8.0</v>
+      </c>
+      <c r="C5" s="24">
+        <v>8.0</v>
+      </c>
       <c r="D5" s="24">
         <v>0.0</v>
       </c>
       <c r="E5" s="25">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="22" t="s">
         <v>11</v>
       </c>
+      <c r="B6" s="22">
+        <v>36.0</v>
+      </c>
+      <c r="C6" s="22">
+        <v>9.0</v>
+      </c>
+      <c r="D6" s="22">
+        <v>0.0</v>
+      </c>
       <c r="E6" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="F6" s="23">
+        <f>SUM(E6:E9)</f>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="22" t="s">
         <v>7</v>
       </c>
+      <c r="B7" s="22">
+        <v>14.0</v>
+      </c>
+      <c r="C7" s="22">
+        <v>13.0</v>
+      </c>
       <c r="D7" s="22">
         <v>0.0</v>
       </c>
       <c r="E7" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="22" t="s">
         <v>13</v>
       </c>
+      <c r="B8" s="22">
+        <v>19.0</v>
+      </c>
+      <c r="C8" s="22">
+        <v>9.0</v>
+      </c>
       <c r="D8" s="22">
         <v>0.0</v>
       </c>
       <c r="E8" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="22" t="s">
         <v>17</v>
       </c>
+      <c r="B9" s="22">
+        <v>12.0</v>
+      </c>
+      <c r="C9" s="22">
+        <v>4.0</v>
+      </c>
       <c r="D9" s="22">
         <v>0.0</v>
       </c>
       <c r="E9" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2421,6 +2498,9 @@
       <c r="E1" s="22" t="s">
         <v>56</v>
       </c>
+      <c r="F1" s="22" t="s">
+        <v>68</v>
+      </c>
       <c r="G1" s="22" t="s">
         <v>21</v>
       </c>
@@ -2430,11 +2510,24 @@
     </row>
     <row r="2">
       <c r="A2" s="22" t="s">
-        <v>5</v>
+        <v>18</v>
+      </c>
+      <c r="B2" s="22">
+        <v>21.0</v>
+      </c>
+      <c r="C2" s="22">
+        <v>12.0</v>
+      </c>
+      <c r="D2" s="22">
+        <v>0.0</v>
       </c>
       <c r="E2" s="23">
-        <f t="shared" ref="E2:E9" si="1">B2*$H$1 + C2*$H$2 + D2*$H$3</f>
-        <v>0</v>
+        <f t="shared" ref="E2:E9" si="1">ROUND(B2*$H$1 + C2*$H$2 + D2*$H$3,0)</f>
+        <v>2</v>
+      </c>
+      <c r="F2" s="23">
+        <f>SUM(E2:E5)</f>
+        <v>8</v>
       </c>
       <c r="G2" s="22" t="s">
         <v>22</v>
@@ -2445,91 +2538,138 @@
     </row>
     <row r="3">
       <c r="A3" s="22" t="s">
-        <v>18</v>
+        <v>5</v>
+      </c>
+      <c r="B3" s="22">
+        <v>10.0</v>
+      </c>
+      <c r="C3" s="22">
+        <v>10.0</v>
       </c>
       <c r="D3" s="22">
         <v>0.0</v>
       </c>
       <c r="E3" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" s="22" t="s">
         <v>20</v>
       </c>
       <c r="H3" s="22">
-        <v>10.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="22" t="s">
         <v>16</v>
       </c>
+      <c r="B4" s="22">
+        <v>17.0</v>
+      </c>
+      <c r="C4" s="22">
+        <v>9.0</v>
+      </c>
       <c r="D4" s="22">
         <v>0.0</v>
       </c>
       <c r="E4" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
+      <c r="B5" s="24">
+        <v>21.0</v>
+      </c>
+      <c r="C5" s="24">
+        <v>19.0</v>
+      </c>
       <c r="D5" s="24">
         <v>0.0</v>
       </c>
       <c r="E5" s="25">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="22" t="s">
         <v>11</v>
       </c>
+      <c r="B6" s="22">
+        <v>30.0</v>
+      </c>
+      <c r="C6" s="22">
+        <v>19.0</v>
+      </c>
+      <c r="D6" s="22">
+        <v>1.0</v>
+      </c>
       <c r="E6" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="F6" s="23">
+        <f>SUM(E6:E9)</f>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="22" t="s">
         <v>7</v>
       </c>
+      <c r="B7" s="22">
+        <v>13.0</v>
+      </c>
+      <c r="C7" s="22">
+        <v>10.0</v>
+      </c>
       <c r="D7" s="22">
         <v>0.0</v>
       </c>
       <c r="E7" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="22" t="s">
         <v>13</v>
       </c>
+      <c r="B8" s="22">
+        <v>26.0</v>
+      </c>
+      <c r="C8" s="22">
+        <v>10.0</v>
+      </c>
       <c r="D8" s="22">
         <v>0.0</v>
       </c>
       <c r="E8" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="22" t="s">
         <v>17</v>
       </c>
+      <c r="B9" s="22">
+        <v>17.0</v>
+      </c>
+      <c r="C9" s="22">
+        <v>9.0</v>
+      </c>
       <c r="D9" s="22">
         <v>0.0</v>
       </c>
       <c r="E9" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2572,11 +2712,24 @@
     </row>
     <row r="2">
       <c r="A2" s="22" t="s">
-        <v>5</v>
+        <v>18</v>
+      </c>
+      <c r="B2" s="22">
+        <v>24.0</v>
+      </c>
+      <c r="C2" s="22">
+        <v>1.0</v>
+      </c>
+      <c r="D2" s="22">
+        <v>0.0</v>
       </c>
       <c r="E2" s="23">
-        <f t="shared" ref="E2:E9" si="1">B2*$H$1 + C2*$H$2 + D2*$H$3</f>
-        <v>0</v>
+        <f t="shared" ref="E2:E9" si="1">ROUND(B2*$H$1 + C2*$H$2 + D2*$H$3,0)</f>
+        <v>2</v>
+      </c>
+      <c r="F2" s="23">
+        <f>SUM(E2:E5)</f>
+        <v>4</v>
       </c>
       <c r="G2" s="22" t="s">
         <v>22</v>
@@ -2587,7 +2740,13 @@
     </row>
     <row r="3">
       <c r="A3" s="22" t="s">
-        <v>18</v>
+        <v>5</v>
+      </c>
+      <c r="B3" s="22">
+        <v>1.0</v>
+      </c>
+      <c r="C3" s="22">
+        <v>1.0</v>
       </c>
       <c r="D3" s="22">
         <v>0.0</v>
@@ -2600,48 +2759,77 @@
         <v>20</v>
       </c>
       <c r="H3" s="22">
-        <v>10.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="22" t="s">
         <v>16</v>
       </c>
+      <c r="B4" s="22">
+        <v>6.0</v>
+      </c>
+      <c r="C4" s="22">
+        <v>0.0</v>
+      </c>
       <c r="D4" s="22">
         <v>0.0</v>
       </c>
       <c r="E4" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
+      <c r="B5" s="24">
+        <v>10.0</v>
+      </c>
+      <c r="C5" s="24">
+        <v>1.0</v>
+      </c>
       <c r="D5" s="24">
         <v>0.0</v>
       </c>
       <c r="E5" s="25">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="22" t="s">
         <v>11</v>
       </c>
+      <c r="B6" s="22">
+        <v>16.0</v>
+      </c>
+      <c r="C6" s="22">
+        <v>0.0</v>
+      </c>
+      <c r="D6" s="22">
+        <v>1.0</v>
+      </c>
       <c r="E6" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="F6" s="23">
+        <f>SUM(E6:E9)</f>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="22" t="s">
         <v>7</v>
       </c>
+      <c r="B7" s="22">
+        <v>2.0</v>
+      </c>
+      <c r="C7" s="22">
+        <v>2.0</v>
+      </c>
       <c r="D7" s="22">
         <v>0.0</v>
       </c>
@@ -2654,24 +2842,36 @@
       <c r="A8" s="22" t="s">
         <v>13</v>
       </c>
+      <c r="B8" s="22">
+        <v>23.0</v>
+      </c>
+      <c r="C8" s="22">
+        <v>0.0</v>
+      </c>
       <c r="D8" s="22">
         <v>0.0</v>
       </c>
       <c r="E8" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="22" t="s">
         <v>17</v>
       </c>
+      <c r="B9" s="22">
+        <v>9.0</v>
+      </c>
+      <c r="C9" s="22">
+        <v>0.0</v>
+      </c>
       <c r="D9" s="22">
         <v>0.0</v>
       </c>
       <c r="E9" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2705,6 +2905,9 @@
       <c r="E1" s="22" t="s">
         <v>56</v>
       </c>
+      <c r="F1" s="22" t="s">
+        <v>68</v>
+      </c>
       <c r="G1" s="22" t="s">
         <v>21</v>
       </c>
@@ -2714,11 +2917,24 @@
     </row>
     <row r="2">
       <c r="A2" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="22">
+        <v>21.0</v>
+      </c>
+      <c r="C2" s="22">
+        <v>5.0</v>
+      </c>
+      <c r="D2" s="22">
+        <v>0.0</v>
+      </c>
+      <c r="E2" s="23">
+        <f t="shared" ref="E2:E9" si="1">ROUND(B2*$H$1 + C2*$H$2 + D2*$H$3,0)</f>
+        <v>2</v>
+      </c>
+      <c r="F2" s="23">
+        <f>SUM(E2:E5)</f>
         <v>5</v>
-      </c>
-      <c r="E2" s="23">
-        <f t="shared" ref="E2:E9" si="1">B2*$H$1 + C2*$H$2 + D2*$H$3</f>
-        <v>0</v>
       </c>
       <c r="G2" s="22" t="s">
         <v>22</v>
@@ -2729,91 +2945,138 @@
     </row>
     <row r="3">
       <c r="A3" s="22" t="s">
-        <v>18</v>
+        <v>5</v>
+      </c>
+      <c r="B3" s="22">
+        <v>5.0</v>
+      </c>
+      <c r="C3" s="22">
+        <v>6.0</v>
       </c>
       <c r="D3" s="22">
         <v>0.0</v>
       </c>
       <c r="E3" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" s="22" t="s">
         <v>20</v>
       </c>
       <c r="H3" s="22">
-        <v>10.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="22" t="s">
         <v>16</v>
       </c>
+      <c r="B4" s="22">
+        <v>7.0</v>
+      </c>
+      <c r="C4" s="22">
+        <v>6.0</v>
+      </c>
       <c r="D4" s="22">
         <v>0.0</v>
       </c>
       <c r="E4" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
+      <c r="B5" s="24">
+        <v>13.0</v>
+      </c>
+      <c r="C5" s="24">
+        <v>7.0</v>
+      </c>
       <c r="D5" s="24">
         <v>0.0</v>
       </c>
       <c r="E5" s="25">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="22" t="s">
         <v>11</v>
       </c>
+      <c r="B6" s="22">
+        <v>23.0</v>
+      </c>
+      <c r="C6" s="22">
+        <v>5.0</v>
+      </c>
+      <c r="D6" s="22">
+        <v>1.0</v>
+      </c>
       <c r="E6" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="F6" s="23">
+        <f>SUM(E6:E9)</f>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="22" t="s">
         <v>7</v>
       </c>
+      <c r="B7" s="22">
+        <v>7.0</v>
+      </c>
+      <c r="C7" s="22">
+        <v>7.0</v>
+      </c>
       <c r="D7" s="22">
         <v>0.0</v>
       </c>
       <c r="E7" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="22" t="s">
         <v>13</v>
       </c>
+      <c r="B8" s="22">
+        <v>14.0</v>
+      </c>
+      <c r="C8" s="22">
+        <v>10.0</v>
+      </c>
       <c r="D8" s="22">
         <v>0.0</v>
       </c>
       <c r="E8" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="22" t="s">
         <v>17</v>
       </c>
+      <c r="B9" s="22">
+        <v>11.0</v>
+      </c>
+      <c r="C9" s="22">
+        <v>3.0</v>
+      </c>
       <c r="D9" s="22">
         <v>0.0</v>
       </c>
       <c r="E9" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>